<commit_message>
feat(students): add enrollment type and bulk import/export functionality
- Add enrollment_type column to students table (regular/irregular)
- Include enrollment type in all CRUD operations and API responses
- Add bulk upsert endpoint for importing students from Excel files
- Add email generation utility for student emails
- Implement Excel export with separate sheets for regular/irregular students
- Add enrollment type filter to student management UI
</commit_message>
<xml_diff>
--- a/assets/list/LIST-OF-ENROLLED-FOR-2ND-SEM-2025-26.xlsx
+++ b/assets/list/LIST-OF-ENROLLED-FOR-2ND-SEM-2025-26.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="12180"/>
+    <workbookView windowWidth="22188" windowHeight="9720" firstSheet="6" activeTab="11"/>
   </bookViews>
   <sheets>
     <sheet name="BTVTED-WFT1" sheetId="1" r:id="rId1"/>
@@ -3111,7 +3111,7 @@
     <t>2023-0176</t>
   </si>
   <si>
-    <t>Romasanta, Patrick James U.</t>
+    <t>Romasanta, Patrick James V.</t>
   </si>
   <si>
     <t>2023-0206</t>
@@ -3485,7 +3485,7 @@
     <numFmt numFmtId="44" formatCode="_-&quot;₱&quot;* #,##0.00_-;\-&quot;₱&quot;* #,##0.00_-;_-&quot;₱&quot;* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="176" formatCode="mmm\-yy"/>
   </numFmts>
-  <fonts count="27">
+  <fonts count="26">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3530,13 +3530,6 @@
       <color theme="1"/>
       <name val="Arial"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <u/>
@@ -4026,28 +4019,31 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -4056,118 +4052,115 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -4385,8 +4378,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="779145" y="0"/>
-          <a:ext cx="4357370" cy="967740"/>
+          <a:off x="792480" y="0"/>
+          <a:ext cx="4479925" cy="967740"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4432,8 +4425,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="992505" y="0"/>
-          <a:ext cx="4349115" cy="1116330"/>
+          <a:off x="1005840" y="0"/>
+          <a:ext cx="4480560" cy="944880"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4479,8 +4472,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="765175" y="0"/>
-          <a:ext cx="4348480" cy="1077595"/>
+          <a:off x="778510" y="0"/>
+          <a:ext cx="4477385" cy="940435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4526,8 +4519,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="741045" y="22860"/>
-          <a:ext cx="4351655" cy="1104265"/>
+          <a:off x="754380" y="22860"/>
+          <a:ext cx="4482465" cy="932815"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4573,8 +4566,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="862965" y="0"/>
-          <a:ext cx="4347210" cy="1122045"/>
+          <a:off x="876300" y="0"/>
+          <a:ext cx="4475480" cy="950595"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4620,8 +4613,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="923925" y="0"/>
-          <a:ext cx="4349750" cy="1120775"/>
+          <a:off x="937260" y="0"/>
+          <a:ext cx="4476750" cy="949325"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4667,8 +4660,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="718185" y="0"/>
-          <a:ext cx="4354195" cy="1116330"/>
+          <a:off x="731520" y="0"/>
+          <a:ext cx="4480560" cy="944880"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4714,8 +4707,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="779145" y="0"/>
-          <a:ext cx="4356100" cy="1082040"/>
+          <a:off x="792480" y="0"/>
+          <a:ext cx="4484370" cy="944880"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4761,8 +4754,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="878205" y="0"/>
-          <a:ext cx="4351655" cy="1116330"/>
+          <a:off x="891540" y="0"/>
+          <a:ext cx="4480560" cy="944880"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4808,8 +4801,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="802005" y="0"/>
-          <a:ext cx="4364355" cy="1116330"/>
+          <a:off x="815340" y="0"/>
+          <a:ext cx="4480560" cy="944880"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4855,8 +4848,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="802005" y="0"/>
-          <a:ext cx="4352925" cy="1116330"/>
+          <a:off x="815340" y="0"/>
+          <a:ext cx="4480560" cy="944880"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4902,8 +4895,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="923925" y="0"/>
-          <a:ext cx="4348480" cy="1084580"/>
+          <a:off x="937260" y="0"/>
+          <a:ext cx="4481195" cy="947420"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4949,8 +4942,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1053465" y="0"/>
-          <a:ext cx="4335780" cy="1121410"/>
+          <a:off x="1066800" y="0"/>
+          <a:ext cx="4465320" cy="949960"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4996,8 +4989,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="710565" y="0"/>
-          <a:ext cx="4350385" cy="1118870"/>
+          <a:off x="723900" y="0"/>
+          <a:ext cx="4478020" cy="947420"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5268,15 +5261,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A5:I61"/>
-  <sheetFormatPr defaultColWidth="33.8857142857143" defaultRowHeight="16.05" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="33.8888888888889" defaultRowHeight="16.05" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="7" style="36" customWidth="1"/>
-    <col min="2" max="2" width="24.8857142857143" style="37" customWidth="1"/>
-    <col min="3" max="3" width="14.8857142857143" style="36" customWidth="1"/>
+    <col min="2" max="2" width="24.8888888888889" style="37" customWidth="1"/>
+    <col min="3" max="3" width="14.8888888888889" style="36" customWidth="1"/>
     <col min="4" max="4" width="14" style="36" customWidth="1"/>
-    <col min="5" max="5" width="10.4380952380952" style="36" customWidth="1"/>
-    <col min="6" max="6" width="16.1047619047619" style="36" customWidth="1"/>
-    <col min="7" max="16384" width="33.8857142857143" style="36"/>
+    <col min="5" max="5" width="10.4351851851852" style="36" customWidth="1"/>
+    <col min="6" max="6" width="16.1018518518519" style="36" customWidth="1"/>
+    <col min="7" max="16384" width="33.8888888888889" style="36"/>
   </cols>
   <sheetData>
     <row r="5" ht="25.2" customHeight="1"/>
@@ -6045,15 +6038,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A7:H48"/>
-  <sheetFormatPr defaultColWidth="28.2190476190476" defaultRowHeight="16.5" outlineLevelCol="7"/>
+  <sheetFormatPr defaultColWidth="28.2222222222222" defaultRowHeight="13.8" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="7" style="1" customWidth="1"/>
-    <col min="2" max="2" width="24.8857142857143" style="2" customWidth="1"/>
+    <col min="2" max="2" width="24.8888888888889" style="2" customWidth="1"/>
     <col min="3" max="3" width="16" style="3" customWidth="1"/>
-    <col min="4" max="4" width="14.8857142857143" style="3" customWidth="1"/>
-    <col min="5" max="5" width="12.8857142857143" style="3" customWidth="1"/>
-    <col min="6" max="6" width="10.8857142857143" style="4" customWidth="1"/>
-    <col min="7" max="16384" width="28.2190476190476" style="3"/>
+    <col min="4" max="4" width="14.8888888888889" style="3" customWidth="1"/>
+    <col min="5" max="5" width="12.8888888888889" style="3" customWidth="1"/>
+    <col min="6" max="6" width="10.8888888888889" style="4" customWidth="1"/>
+    <col min="7" max="16384" width="28.2222222222222" style="3"/>
   </cols>
   <sheetData>
     <row r="7" ht="16.05" customHeight="1" spans="1:6">
@@ -6676,15 +6669,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A5:H49"/>
-  <sheetFormatPr defaultColWidth="28.2190476190476" defaultRowHeight="16.5" outlineLevelCol="7"/>
+  <sheetFormatPr defaultColWidth="28.2222222222222" defaultRowHeight="13.8" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="7" style="1" customWidth="1"/>
-    <col min="2" max="2" width="26.4380952380952" style="2" customWidth="1"/>
+    <col min="2" max="2" width="26.4351851851852" style="2" customWidth="1"/>
     <col min="3" max="3" width="16" style="3" customWidth="1"/>
-    <col min="4" max="4" width="13.1047619047619" style="3" customWidth="1"/>
+    <col min="4" max="4" width="13.1018518518519" style="3" customWidth="1"/>
     <col min="5" max="5" width="12.3333333333333" style="3" customWidth="1"/>
     <col min="6" max="6" width="12" style="4" customWidth="1"/>
-    <col min="7" max="16384" width="28.2190476190476" style="3"/>
+    <col min="7" max="16384" width="28.2222222222222" style="3"/>
   </cols>
   <sheetData>
     <row r="5" ht="28.8" customHeight="1"/>
@@ -7488,15 +7481,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A7:F53"/>
-  <sheetFormatPr defaultColWidth="28.2190476190476" defaultRowHeight="16.5" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="28.2222222222222" defaultRowHeight="13.8" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="7" style="1" customWidth="1"/>
-    <col min="2" max="2" width="29.552380952381" style="2" customWidth="1"/>
-    <col min="3" max="3" width="13.8857142857143" style="3" customWidth="1"/>
+    <col min="2" max="2" width="29.5555555555556" style="2" customWidth="1"/>
+    <col min="3" max="3" width="13.8888888888889" style="3" customWidth="1"/>
     <col min="4" max="4" width="13.6666666666667" style="3" customWidth="1"/>
-    <col min="5" max="5" width="11.2190476190476" style="3" customWidth="1"/>
-    <col min="6" max="6" width="11.552380952381" style="4" customWidth="1"/>
-    <col min="7" max="16384" width="28.2190476190476" style="3"/>
+    <col min="5" max="5" width="11.2222222222222" style="3" customWidth="1"/>
+    <col min="6" max="6" width="11.5555555555556" style="4" customWidth="1"/>
+    <col min="7" max="16384" width="28.2222222222222" style="3"/>
   </cols>
   <sheetData>
     <row r="7" ht="16.05" customHeight="1" spans="1:6">
@@ -8369,15 +8362,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A7:F41"/>
-  <sheetFormatPr defaultColWidth="28.2190476190476" defaultRowHeight="16.5" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="28.2222222222222" defaultRowHeight="13.8" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="7" style="1" customWidth="1"/>
-    <col min="2" max="2" width="24.8857142857143" style="2" customWidth="1"/>
+    <col min="2" max="2" width="24.8888888888889" style="2" customWidth="1"/>
     <col min="3" max="3" width="16" style="3" customWidth="1"/>
     <col min="4" max="4" width="13.3333333333333" style="3" customWidth="1"/>
-    <col min="5" max="5" width="12.8857142857143" style="3" customWidth="1"/>
-    <col min="6" max="6" width="13.2190476190476" style="4" customWidth="1"/>
-    <col min="7" max="16384" width="28.2190476190476" style="3"/>
+    <col min="5" max="5" width="12.8888888888889" style="3" customWidth="1"/>
+    <col min="6" max="6" width="13.2222222222222" style="4" customWidth="1"/>
+    <col min="7" max="16384" width="28.2222222222222" style="3"/>
   </cols>
   <sheetData>
     <row r="7" ht="16.05" customHeight="1" spans="1:6">
@@ -8966,15 +8959,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A7:F48"/>
-  <sheetFormatPr defaultColWidth="28.2190476190476" defaultRowHeight="16.5" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="28.2222222222222" defaultRowHeight="13.8" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="7" style="1" customWidth="1"/>
-    <col min="2" max="2" width="22.7809523809524" style="2" customWidth="1"/>
+    <col min="2" max="2" width="22.7777777777778" style="2" customWidth="1"/>
     <col min="3" max="3" width="16" style="3" customWidth="1"/>
-    <col min="4" max="4" width="14.8857142857143" style="3" customWidth="1"/>
-    <col min="5" max="5" width="12.8857142857143" style="3" customWidth="1"/>
-    <col min="6" max="6" width="13.2190476190476" style="4" customWidth="1"/>
-    <col min="7" max="16384" width="28.2190476190476" style="3"/>
+    <col min="4" max="4" width="14.8888888888889" style="3" customWidth="1"/>
+    <col min="5" max="5" width="12.8888888888889" style="3" customWidth="1"/>
+    <col min="6" max="6" width="13.2222222222222" style="4" customWidth="1"/>
+    <col min="7" max="16384" width="28.2222222222222" style="3"/>
   </cols>
   <sheetData>
     <row r="7" ht="16.05" customHeight="1" spans="1:6">
@@ -9611,15 +9604,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A6:F50"/>
-  <sheetFormatPr defaultColWidth="28.2190476190476" defaultRowHeight="16.5" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="28.2222222222222" defaultRowHeight="13.8" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="7" style="36" customWidth="1"/>
-    <col min="2" max="2" width="24.7809523809524" style="37" customWidth="1"/>
-    <col min="3" max="3" width="14.552380952381" style="36" customWidth="1"/>
-    <col min="4" max="4" width="13.552380952381" style="36" customWidth="1"/>
-    <col min="5" max="5" width="13.2190476190476" style="36" customWidth="1"/>
+    <col min="2" max="2" width="24.7777777777778" style="37" customWidth="1"/>
+    <col min="3" max="3" width="14.5555555555556" style="36" customWidth="1"/>
+    <col min="4" max="4" width="13.5555555555556" style="36" customWidth="1"/>
+    <col min="5" max="5" width="13.2222222222222" style="36" customWidth="1"/>
     <col min="6" max="6" width="13" style="36" customWidth="1"/>
-    <col min="7" max="16384" width="28.2190476190476" style="36"/>
+    <col min="7" max="16384" width="28.2222222222222" style="36"/>
   </cols>
   <sheetData>
     <row r="6" ht="20.4" customHeight="1"/>
@@ -10407,15 +10400,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A5:H60"/>
-  <sheetFormatPr defaultColWidth="28.2190476190476" defaultRowHeight="16.5" outlineLevelCol="7"/>
+  <sheetFormatPr defaultColWidth="28.2222222222222" defaultRowHeight="13.8" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="7" style="3" customWidth="1"/>
-    <col min="2" max="2" width="26.4380952380952" style="2" customWidth="1"/>
+    <col min="2" max="2" width="26.4351851851852" style="2" customWidth="1"/>
     <col min="3" max="3" width="16" style="3" customWidth="1"/>
     <col min="4" max="4" width="14.3333333333333" style="3" customWidth="1"/>
     <col min="5" max="5" width="10.6666666666667" style="3" customWidth="1"/>
-    <col min="6" max="6" width="13.2190476190476" style="4" customWidth="1"/>
-    <col min="7" max="16384" width="28.2190476190476" style="3"/>
+    <col min="6" max="6" width="13.2222222222222" style="4" customWidth="1"/>
+    <col min="7" max="16384" width="28.2222222222222" style="3"/>
   </cols>
   <sheetData>
     <row r="5" ht="28.8" customHeight="1"/>
@@ -11406,15 +11399,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A7:F69"/>
-  <sheetFormatPr defaultColWidth="28.2190476190476" defaultRowHeight="16.5" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="28.2222222222222" defaultRowHeight="13.8" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="7" style="3" customWidth="1"/>
-    <col min="2" max="2" width="24.8857142857143" style="2" customWidth="1"/>
+    <col min="2" max="2" width="24.8888888888889" style="2" customWidth="1"/>
     <col min="3" max="3" width="16" style="3" customWidth="1"/>
-    <col min="4" max="4" width="14.8857142857143" style="3" customWidth="1"/>
-    <col min="5" max="5" width="11.7809523809524" style="3" customWidth="1"/>
-    <col min="6" max="6" width="13.2190476190476" style="4" customWidth="1"/>
-    <col min="7" max="16384" width="28.2190476190476" style="3"/>
+    <col min="4" max="4" width="14.8888888888889" style="3" customWidth="1"/>
+    <col min="5" max="5" width="11.7777777777778" style="3" customWidth="1"/>
+    <col min="6" max="6" width="13.2222222222222" style="4" customWidth="1"/>
+    <col min="7" max="16384" width="28.2222222222222" style="3"/>
   </cols>
   <sheetData>
     <row r="7" ht="16.05" customHeight="1" spans="1:6">
@@ -12530,15 +12523,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A7:F48"/>
-  <sheetFormatPr defaultColWidth="28.2190476190476" defaultRowHeight="16.5" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="28.2222222222222" defaultRowHeight="13.8" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="7" style="1" customWidth="1"/>
-    <col min="2" max="2" width="24.8857142857143" style="2" customWidth="1"/>
+    <col min="2" max="2" width="24.8888888888889" style="2" customWidth="1"/>
     <col min="3" max="3" width="13" style="3" customWidth="1"/>
-    <col min="4" max="4" width="9.78095238095238" style="3" customWidth="1"/>
-    <col min="5" max="5" width="13.2190476190476" style="3" customWidth="1"/>
-    <col min="6" max="6" width="17.4380952380952" style="4" customWidth="1"/>
-    <col min="7" max="16384" width="28.2190476190476" style="3"/>
+    <col min="4" max="4" width="9.77777777777778" style="3" customWidth="1"/>
+    <col min="5" max="5" width="13.2222222222222" style="3" customWidth="1"/>
+    <col min="6" max="6" width="17.4351851851852" style="4" customWidth="1"/>
+    <col min="7" max="16384" width="28.2222222222222" style="3"/>
   </cols>
   <sheetData>
     <row r="7" ht="16.05" customHeight="1" spans="1:6">
@@ -13303,15 +13296,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A7:F40"/>
-  <sheetFormatPr defaultColWidth="28.2190476190476" defaultRowHeight="16.5" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="28.2222222222222" defaultRowHeight="13.8" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="7" style="1" customWidth="1"/>
     <col min="2" max="2" width="24.6666666666667" style="2" customWidth="1"/>
-    <col min="3" max="3" width="13.8857142857143" style="3" customWidth="1"/>
-    <col min="4" max="4" width="14.8857142857143" style="3" customWidth="1"/>
-    <col min="5" max="5" width="13.2190476190476" style="3" customWidth="1"/>
-    <col min="6" max="6" width="13.2190476190476" style="4" customWidth="1"/>
-    <col min="7" max="16384" width="28.2190476190476" style="3"/>
+    <col min="3" max="3" width="13.8888888888889" style="3" customWidth="1"/>
+    <col min="4" max="4" width="14.8888888888889" style="3" customWidth="1"/>
+    <col min="5" max="5" width="13.2222222222222" style="3" customWidth="1"/>
+    <col min="6" max="6" width="13.2222222222222" style="4" customWidth="1"/>
+    <col min="7" max="16384" width="28.2222222222222" style="3"/>
   </cols>
   <sheetData>
     <row r="7" ht="16.05" customHeight="1" spans="1:6">
@@ -13889,15 +13882,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A5:H65"/>
-  <sheetFormatPr defaultColWidth="28.2190476190476" defaultRowHeight="16.5" outlineLevelCol="7"/>
+  <sheetFormatPr defaultColWidth="28.2222222222222" defaultRowHeight="13.8" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="7" style="1" customWidth="1"/>
-    <col min="2" max="2" width="26.4380952380952" style="2" customWidth="1"/>
+    <col min="2" max="2" width="26.4351851851852" style="2" customWidth="1"/>
     <col min="3" max="3" width="16" style="3" customWidth="1"/>
-    <col min="4" max="4" width="14.8857142857143" style="3" customWidth="1"/>
+    <col min="4" max="4" width="14.8888888888889" style="3" customWidth="1"/>
     <col min="5" max="5" width="12.3333333333333" style="3" customWidth="1"/>
     <col min="6" max="6" width="10.3333333333333" style="4" customWidth="1"/>
-    <col min="7" max="16384" width="28.2190476190476" style="3"/>
+    <col min="7" max="16384" width="28.2222222222222" style="3"/>
   </cols>
   <sheetData>
     <row r="5" ht="28.8" customHeight="1"/>
@@ -14999,15 +14992,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A7:G64"/>
-  <sheetFormatPr defaultColWidth="28.2190476190476" defaultRowHeight="16.5" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="28.2222222222222" defaultRowHeight="13.8" outlineLevelCol="6"/>
   <cols>
     <col min="1" max="1" width="7" style="1" customWidth="1"/>
     <col min="2" max="2" width="27" style="2" customWidth="1"/>
     <col min="3" max="3" width="16" style="3" customWidth="1"/>
     <col min="4" max="4" width="13.6666666666667" style="3" customWidth="1"/>
-    <col min="5" max="5" width="11.2190476190476" style="3" customWidth="1"/>
-    <col min="6" max="6" width="11.552380952381" style="4" customWidth="1"/>
-    <col min="7" max="16384" width="28.2190476190476" style="3"/>
+    <col min="5" max="5" width="11.2222222222222" style="3" customWidth="1"/>
+    <col min="6" max="6" width="11.5555555555556" style="4" customWidth="1"/>
+    <col min="7" max="16384" width="28.2222222222222" style="3"/>
   </cols>
   <sheetData>
     <row r="7" ht="16.05" customHeight="1" spans="1:6">
@@ -16088,14 +16081,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A7:F46"/>
-  <sheetFormatPr defaultColWidth="28.2190476190476" defaultRowHeight="16.5" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="28.2222222222222" defaultRowHeight="13.8" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="7" style="1" customWidth="1"/>
-    <col min="2" max="2" width="24.8857142857143" style="2" customWidth="1"/>
+    <col min="2" max="2" width="24.8888888888889" style="2" customWidth="1"/>
     <col min="3" max="3" width="16" style="3" customWidth="1"/>
-    <col min="4" max="5" width="12.8857142857143" style="3" customWidth="1"/>
-    <col min="6" max="6" width="13.2190476190476" style="4" customWidth="1"/>
-    <col min="7" max="16384" width="28.2190476190476" style="3"/>
+    <col min="4" max="5" width="12.8888888888889" style="3" customWidth="1"/>
+    <col min="6" max="6" width="13.2222222222222" style="4" customWidth="1"/>
+    <col min="7" max="16384" width="28.2222222222222" style="3"/>
   </cols>
   <sheetData>
     <row r="7" ht="16.05" customHeight="1" spans="1:6">

</xml_diff>